<commit_message>
Se modifico el algoritmo para que tomara en cuenta el horario de los lugares y el tiempo de regreso a la base al final de la ruta
</commit_message>
<xml_diff>
--- a/TSOoficios/BD Registros.xlsx
+++ b/TSOoficios/BD Registros.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moral\Desktop\TSOoficios\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\moral\Desktop\TSOPIA\TSOoficios\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{410B0DCD-80A5-4E5A-9911-490011B4E360}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B007033E-AE89-4168-BEA3-83736F9BFA98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56,7 +56,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="804" uniqueCount="106">
   <si>
     <t>Día</t>
   </si>
@@ -368,6 +368,12 @@
   </si>
   <si>
     <t>total</t>
+  </si>
+  <si>
+    <t>HoraCierre</t>
+  </si>
+  <si>
+    <t>HoraApertura</t>
   </si>
 </sst>
 </file>
@@ -519,7 +525,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
@@ -552,6 +558,10 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="20" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="20" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -856,15 +866,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:L638"/>
+  <dimension ref="A1:M638"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="2" max="2" width="19" customWidth="1"/>
     <col min="3" max="3" width="20.7265625" customWidth="1"/>
     <col min="4" max="4" width="70.7265625" customWidth="1"/>
-    <col min="5" max="5" width="87.1796875" customWidth="1"/>
+    <col min="5" max="5" width="100.81640625" customWidth="1"/>
     <col min="6" max="6" width="23.7265625" customWidth="1"/>
-    <col min="7" max="7" width="12.81640625" customWidth="1"/>
+    <col min="7" max="7" width="18.54296875" customWidth="1"/>
     <col min="8" max="8" width="20.453125" customWidth="1"/>
     <col min="9" max="9" width="15.1796875" customWidth="1"/>
     <col min="10" max="10" width="32" customWidth="1"/>
@@ -873,7 +883,7 @@
     <col min="13" max="13" width="11.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -890,28 +900,31 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
+        <v>105</v>
       </c>
       <c r="G1" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="H1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="I1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="J1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>1</v>
       </c>
@@ -925,20 +938,23 @@
       <c r="E2" t="s">
         <v>95</v>
       </c>
-      <c r="F2" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="G2" t="s">
+      <c r="F2" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G2" s="16">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="H2" t="s">
         <v>52</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>98</v>
       </c>
-      <c r="J2" s="13">
+      <c r="K2" s="13">
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1</v>
       </c>
@@ -954,29 +970,32 @@
       <c r="E3" t="s">
         <v>30</v>
       </c>
-      <c r="F3" t="s">
-        <v>47</v>
-      </c>
-      <c r="G3" t="s">
-        <v>51</v>
+      <c r="F3" s="16">
+        <v>0</v>
+      </c>
+      <c r="G3" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H3" t="s">
+        <v>51</v>
+      </c>
+      <c r="I3" t="s">
         <v>75</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>72</v>
       </c>
-      <c r="J3" s="13">
+      <c r="K3" s="13">
         <v>40</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>73</v>
       </c>
-      <c r="L3" t="s">
+      <c r="M3" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1</v>
       </c>
@@ -992,29 +1011,32 @@
       <c r="E4" t="s">
         <v>31</v>
       </c>
-      <c r="F4" t="s">
-        <v>47</v>
-      </c>
-      <c r="G4" t="s">
+      <c r="F4" s="16">
+        <v>0</v>
+      </c>
+      <c r="G4" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H4" t="s">
         <v>52</v>
       </c>
-      <c r="H4" t="s">
+      <c r="I4" t="s">
         <v>75</v>
       </c>
-      <c r="I4" t="s">
+      <c r="J4" t="s">
         <v>72</v>
       </c>
-      <c r="J4" s="13">
+      <c r="K4" s="13">
         <v>25</v>
       </c>
-      <c r="K4" t="s">
+      <c r="L4" t="s">
         <v>73</v>
       </c>
-      <c r="L4" t="s">
+      <c r="M4" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1</v>
       </c>
@@ -1030,29 +1052,32 @@
       <c r="E5" t="s">
         <v>32</v>
       </c>
-      <c r="F5" t="s">
-        <v>47</v>
-      </c>
-      <c r="G5" t="s">
-        <v>51</v>
+      <c r="F5" s="16">
+        <v>0</v>
+      </c>
+      <c r="G5" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H5" t="s">
+        <v>51</v>
+      </c>
+      <c r="I5" t="s">
         <v>75</v>
       </c>
-      <c r="I5" t="s">
+      <c r="J5" t="s">
         <v>72</v>
       </c>
-      <c r="J5" s="13">
-        <v>0</v>
-      </c>
-      <c r="K5" t="s">
+      <c r="K5" s="13">
+        <v>0</v>
+      </c>
+      <c r="L5" t="s">
         <v>73</v>
       </c>
-      <c r="L5" t="s">
+      <c r="M5" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1</v>
       </c>
@@ -1068,29 +1093,32 @@
       <c r="E6" t="s">
         <v>32</v>
       </c>
-      <c r="F6" t="s">
-        <v>47</v>
-      </c>
-      <c r="G6" t="s">
-        <v>51</v>
+      <c r="F6" s="16">
+        <v>0</v>
+      </c>
+      <c r="G6" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H6" t="s">
+        <v>51</v>
+      </c>
+      <c r="I6" t="s">
         <v>75</v>
       </c>
-      <c r="I6" t="s">
+      <c r="J6" t="s">
         <v>72</v>
       </c>
-      <c r="J6" s="13">
+      <c r="K6" s="13">
         <v>25</v>
       </c>
-      <c r="K6" t="s">
+      <c r="L6" t="s">
         <v>73</v>
       </c>
-      <c r="L6" t="s">
+      <c r="M6" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1</v>
       </c>
@@ -1106,29 +1134,32 @@
       <c r="E7" t="s">
         <v>30</v>
       </c>
-      <c r="F7" t="s">
-        <v>47</v>
-      </c>
-      <c r="G7" t="s">
-        <v>51</v>
+      <c r="F7" s="16">
+        <v>0</v>
+      </c>
+      <c r="G7" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H7" t="s">
+        <v>51</v>
+      </c>
+      <c r="I7" t="s">
         <v>75</v>
       </c>
-      <c r="I7" t="s">
+      <c r="J7" t="s">
         <v>72</v>
       </c>
-      <c r="J7" s="13">
+      <c r="K7" s="13">
         <v>30</v>
       </c>
-      <c r="K7" t="s">
+      <c r="L7" t="s">
         <v>73</v>
       </c>
-      <c r="L7" t="s">
+      <c r="M7" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1</v>
       </c>
@@ -1144,29 +1175,32 @@
       <c r="E8" t="s">
         <v>33</v>
       </c>
-      <c r="F8" t="s">
-        <v>48</v>
-      </c>
-      <c r="G8" t="s">
-        <v>51</v>
+      <c r="F8" s="16">
+        <v>0.375</v>
+      </c>
+      <c r="G8" s="16">
+        <v>0.70833333333333337</v>
       </c>
       <c r="H8" t="s">
+        <v>51</v>
+      </c>
+      <c r="I8" t="s">
         <v>76</v>
       </c>
-      <c r="I8" t="s">
+      <c r="J8" t="s">
         <v>73</v>
       </c>
-      <c r="J8" s="13">
+      <c r="K8" s="13">
         <v>20</v>
       </c>
-      <c r="K8" t="s">
+      <c r="L8" t="s">
         <v>73</v>
       </c>
-      <c r="L8" t="s">
+      <c r="M8" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1</v>
       </c>
@@ -1182,29 +1216,32 @@
       <c r="E9" t="s">
         <v>34</v>
       </c>
-      <c r="F9" t="s">
-        <v>47</v>
-      </c>
-      <c r="G9" t="s">
+      <c r="F9" s="16">
+        <v>0</v>
+      </c>
+      <c r="G9" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H9" t="s">
         <v>52</v>
       </c>
-      <c r="H9" t="s">
+      <c r="I9" t="s">
         <v>75</v>
       </c>
-      <c r="I9" t="s">
+      <c r="J9" t="s">
         <v>72</v>
       </c>
-      <c r="J9" s="13">
+      <c r="K9" s="13">
         <v>15</v>
       </c>
-      <c r="K9" t="s">
+      <c r="L9" t="s">
         <v>73</v>
       </c>
-      <c r="L9" t="s">
+      <c r="M9" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1</v>
       </c>
@@ -1220,29 +1257,32 @@
       <c r="E10" t="s">
         <v>35</v>
       </c>
-      <c r="F10" t="s">
-        <v>47</v>
-      </c>
-      <c r="G10" t="s">
-        <v>51</v>
+      <c r="F10" s="16">
+        <v>0</v>
+      </c>
+      <c r="G10" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H10" t="s">
+        <v>51</v>
+      </c>
+      <c r="I10" t="s">
         <v>75</v>
       </c>
-      <c r="I10" t="s">
+      <c r="J10" t="s">
         <v>72</v>
       </c>
-      <c r="J10" s="13">
+      <c r="K10" s="13">
         <v>25</v>
       </c>
-      <c r="K10" t="s">
+      <c r="L10" t="s">
         <v>73</v>
       </c>
-      <c r="L10" t="s">
+      <c r="M10" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1</v>
       </c>
@@ -1258,29 +1298,32 @@
       <c r="E11" t="s">
         <v>36</v>
       </c>
-      <c r="F11" t="s">
-        <v>47</v>
-      </c>
-      <c r="G11" t="s">
-        <v>51</v>
+      <c r="F11" s="16">
+        <v>0</v>
+      </c>
+      <c r="G11" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H11" t="s">
+        <v>51</v>
+      </c>
+      <c r="I11" t="s">
         <v>75</v>
       </c>
-      <c r="I11" t="s">
+      <c r="J11" t="s">
         <v>72</v>
       </c>
-      <c r="J11" s="13">
+      <c r="K11" s="13">
         <v>20</v>
       </c>
-      <c r="K11" t="s">
+      <c r="L11" t="s">
         <v>73</v>
       </c>
-      <c r="L11" t="s">
+      <c r="M11" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>1</v>
       </c>
@@ -1296,29 +1339,32 @@
       <c r="E12" t="s">
         <v>37</v>
       </c>
-      <c r="F12" t="s">
-        <v>49</v>
-      </c>
-      <c r="G12" t="s">
-        <v>51</v>
+      <c r="F12" s="16">
+        <v>0.375</v>
+      </c>
+      <c r="G12" s="16">
+        <v>0.70833333333333337</v>
       </c>
       <c r="H12" t="s">
+        <v>51</v>
+      </c>
+      <c r="I12" t="s">
         <v>76</v>
       </c>
-      <c r="I12" t="s">
+      <c r="J12" t="s">
         <v>73</v>
       </c>
-      <c r="J12" s="13">
+      <c r="K12" s="13">
         <v>40</v>
       </c>
-      <c r="K12" t="s">
+      <c r="L12" t="s">
         <v>73</v>
       </c>
-      <c r="L12" t="s">
+      <c r="M12" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1</v>
       </c>
@@ -1334,29 +1380,32 @@
       <c r="E13" t="s">
         <v>38</v>
       </c>
-      <c r="F13" t="s">
-        <v>47</v>
-      </c>
-      <c r="G13" t="s">
+      <c r="F13" s="16">
+        <v>0</v>
+      </c>
+      <c r="G13" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H13" t="s">
         <v>53</v>
       </c>
-      <c r="H13" t="s">
+      <c r="I13" t="s">
         <v>76</v>
       </c>
-      <c r="I13" t="s">
+      <c r="J13" t="s">
         <v>72</v>
       </c>
-      <c r="J13" s="13">
+      <c r="K13" s="13">
         <v>30</v>
       </c>
-      <c r="K13" t="s">
+      <c r="L13" t="s">
         <v>73</v>
       </c>
-      <c r="L13" t="s">
+      <c r="M13" t="s">
         <v>78</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1</v>
       </c>
@@ -1372,29 +1421,32 @@
       <c r="E14" t="s">
         <v>39</v>
       </c>
-      <c r="F14" t="s">
-        <v>47</v>
-      </c>
-      <c r="G14" t="s">
-        <v>51</v>
+      <c r="F14" s="16">
+        <v>0</v>
+      </c>
+      <c r="G14" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H14" t="s">
+        <v>51</v>
+      </c>
+      <c r="I14" t="s">
         <v>75</v>
       </c>
-      <c r="I14" t="s">
+      <c r="J14" t="s">
         <v>72</v>
       </c>
-      <c r="J14" s="13">
+      <c r="K14" s="13">
         <v>30</v>
       </c>
-      <c r="K14" t="s">
+      <c r="L14" t="s">
         <v>73</v>
       </c>
-      <c r="L14" t="s">
+      <c r="M14" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1</v>
       </c>
@@ -1410,29 +1462,32 @@
       <c r="E15" t="s">
         <v>38</v>
       </c>
-      <c r="F15" t="s">
-        <v>47</v>
-      </c>
-      <c r="G15" t="s">
+      <c r="F15" s="16">
+        <v>0</v>
+      </c>
+      <c r="G15" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H15" t="s">
         <v>53</v>
       </c>
-      <c r="H15" t="s">
+      <c r="I15" t="s">
         <v>75</v>
       </c>
-      <c r="I15" t="s">
+      <c r="J15" t="s">
         <v>72</v>
       </c>
-      <c r="J15" s="13">
-        <v>0</v>
-      </c>
-      <c r="K15" t="s">
+      <c r="K15" s="13">
+        <v>0</v>
+      </c>
+      <c r="L15" t="s">
         <v>73</v>
       </c>
-      <c r="L15" t="s">
+      <c r="M15" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1</v>
       </c>
@@ -1448,29 +1503,32 @@
       <c r="E16" t="s">
         <v>38</v>
       </c>
-      <c r="F16" t="s">
-        <v>47</v>
-      </c>
-      <c r="G16" t="s">
+      <c r="F16" s="16">
+        <v>0</v>
+      </c>
+      <c r="G16" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H16" t="s">
         <v>53</v>
       </c>
-      <c r="H16" t="s">
+      <c r="I16" t="s">
         <v>75</v>
       </c>
-      <c r="I16" t="s">
+      <c r="J16" t="s">
         <v>72</v>
       </c>
-      <c r="J16" s="13">
+      <c r="K16" s="13">
         <v>20</v>
       </c>
-      <c r="K16" t="s">
+      <c r="L16" t="s">
         <v>73</v>
       </c>
-      <c r="L16" t="s">
+      <c r="M16" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1</v>
       </c>
@@ -1486,29 +1544,32 @@
       <c r="E17" t="s">
         <v>40</v>
       </c>
-      <c r="F17" t="s">
-        <v>47</v>
-      </c>
-      <c r="G17" t="s">
+      <c r="F17" s="16">
+        <v>0</v>
+      </c>
+      <c r="G17" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H17" t="s">
         <v>53</v>
       </c>
-      <c r="H17" t="s">
+      <c r="I17" t="s">
         <v>75</v>
       </c>
-      <c r="I17" t="s">
+      <c r="J17" t="s">
         <v>72</v>
       </c>
-      <c r="J17" s="13">
+      <c r="K17" s="13">
         <v>70</v>
       </c>
-      <c r="K17" t="s">
+      <c r="L17" t="s">
         <v>73</v>
       </c>
-      <c r="L17" t="s">
+      <c r="M17" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>1</v>
       </c>
@@ -1524,29 +1585,32 @@
       <c r="E18" t="s">
         <v>41</v>
       </c>
-      <c r="F18" t="s">
-        <v>47</v>
-      </c>
-      <c r="G18" t="s">
-        <v>51</v>
+      <c r="F18" s="16">
+        <v>0</v>
+      </c>
+      <c r="G18" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H18" t="s">
+        <v>51</v>
+      </c>
+      <c r="I18" t="s">
         <v>75</v>
       </c>
-      <c r="I18" t="s">
+      <c r="J18" t="s">
         <v>72</v>
       </c>
-      <c r="J18" s="13">
+      <c r="K18" s="13">
         <v>20</v>
       </c>
-      <c r="K18" t="s">
+      <c r="L18" t="s">
         <v>73</v>
       </c>
-      <c r="L18" t="s">
+      <c r="M18" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>1</v>
       </c>
@@ -1562,29 +1626,32 @@
       <c r="E19" t="s">
         <v>42</v>
       </c>
-      <c r="F19" t="s">
-        <v>47</v>
-      </c>
-      <c r="G19" t="s">
+      <c r="F19" s="16">
+        <v>0</v>
+      </c>
+      <c r="G19" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H19" t="s">
         <v>53</v>
       </c>
-      <c r="H19" t="s">
+      <c r="I19" t="s">
         <v>75</v>
       </c>
-      <c r="I19" t="s">
+      <c r="J19" t="s">
         <v>72</v>
       </c>
-      <c r="J19" s="13">
+      <c r="K19" s="13">
         <v>50</v>
       </c>
-      <c r="K19" t="s">
+      <c r="L19" t="s">
         <v>73</v>
       </c>
-      <c r="L19" t="s">
+      <c r="M19" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>1</v>
       </c>
@@ -1600,29 +1667,32 @@
       <c r="E20" t="s">
         <v>43</v>
       </c>
-      <c r="F20" t="s">
-        <v>47</v>
-      </c>
-      <c r="G20" t="s">
-        <v>51</v>
+      <c r="F20" s="16">
+        <v>0</v>
+      </c>
+      <c r="G20" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H20" t="s">
+        <v>51</v>
+      </c>
+      <c r="I20" t="s">
         <v>75</v>
       </c>
-      <c r="I20" t="s">
+      <c r="J20" t="s">
         <v>72</v>
       </c>
-      <c r="J20" s="13">
+      <c r="K20" s="13">
         <v>50</v>
       </c>
-      <c r="K20" t="s">
+      <c r="L20" t="s">
         <v>73</v>
       </c>
-      <c r="L20" t="s">
+      <c r="M20" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>1</v>
       </c>
@@ -1638,29 +1708,32 @@
       <c r="E21" t="s">
         <v>36</v>
       </c>
-      <c r="F21" t="s">
-        <v>47</v>
-      </c>
-      <c r="G21" t="s">
-        <v>51</v>
+      <c r="F21" s="16">
+        <v>0</v>
+      </c>
+      <c r="G21" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H21" t="s">
+        <v>51</v>
+      </c>
+      <c r="I21" t="s">
         <v>75</v>
       </c>
-      <c r="I21" t="s">
+      <c r="J21" t="s">
         <v>72</v>
       </c>
-      <c r="J21" s="13">
+      <c r="K21" s="13">
         <v>30</v>
       </c>
-      <c r="K21" t="s">
+      <c r="L21" t="s">
         <v>73</v>
       </c>
-      <c r="L21" t="s">
+      <c r="M21" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2</v>
       </c>
@@ -1674,20 +1747,23 @@
       <c r="E22" t="s">
         <v>95</v>
       </c>
-      <c r="F22" s="11" t="s">
-        <v>96</v>
-      </c>
-      <c r="G22" t="s">
+      <c r="F22" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G22" s="16">
+        <v>0.70833333333333337</v>
+      </c>
+      <c r="H22" t="s">
         <v>52</v>
       </c>
-      <c r="H22" t="s">
+      <c r="I22" t="s">
         <v>98</v>
       </c>
-      <c r="J22" s="13">
+      <c r="K22" s="13">
         <v>30</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2</v>
       </c>
@@ -1703,29 +1779,32 @@
       <c r="E23" t="s">
         <v>44</v>
       </c>
-      <c r="F23" t="s">
-        <v>47</v>
-      </c>
-      <c r="G23" t="s">
-        <v>51</v>
+      <c r="F23" s="16">
+        <v>0</v>
+      </c>
+      <c r="G23" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H23" t="s">
+        <v>51</v>
+      </c>
+      <c r="I23" t="s">
         <v>75</v>
       </c>
-      <c r="I23" t="s">
+      <c r="J23" t="s">
         <v>72</v>
       </c>
-      <c r="J23" s="13">
+      <c r="K23" s="13">
         <v>30</v>
       </c>
-      <c r="K23" t="s">
+      <c r="L23" t="s">
         <v>73</v>
       </c>
-      <c r="L23" t="s">
+      <c r="M23" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2</v>
       </c>
@@ -1741,29 +1820,32 @@
       <c r="E24" t="s">
         <v>43</v>
       </c>
-      <c r="F24" t="s">
-        <v>47</v>
-      </c>
-      <c r="G24" t="s">
-        <v>51</v>
+      <c r="F24" s="16">
+        <v>0</v>
+      </c>
+      <c r="G24" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H24" t="s">
+        <v>51</v>
+      </c>
+      <c r="I24" t="s">
         <v>75</v>
       </c>
-      <c r="I24" t="s">
+      <c r="J24" t="s">
         <v>72</v>
       </c>
-      <c r="J24" s="13">
+      <c r="K24" s="13">
         <v>40</v>
       </c>
-      <c r="K24" t="s">
+      <c r="L24" t="s">
         <v>73</v>
       </c>
-      <c r="L24" t="s">
+      <c r="M24" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2</v>
       </c>
@@ -1779,29 +1861,32 @@
       <c r="E25" t="s">
         <v>30</v>
       </c>
-      <c r="F25" t="s">
-        <v>47</v>
-      </c>
-      <c r="G25" t="s">
-        <v>51</v>
+      <c r="F25" s="16">
+        <v>0</v>
+      </c>
+      <c r="G25" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H25" t="s">
+        <v>51</v>
+      </c>
+      <c r="I25" t="s">
         <v>75</v>
       </c>
-      <c r="I25" t="s">
+      <c r="J25" t="s">
         <v>72</v>
       </c>
-      <c r="J25" s="13">
+      <c r="K25" s="13">
         <v>40</v>
       </c>
-      <c r="K25" t="s">
+      <c r="L25" t="s">
         <v>73</v>
       </c>
-      <c r="L25" t="s">
+      <c r="M25" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2</v>
       </c>
@@ -1817,29 +1902,32 @@
       <c r="E26" t="s">
         <v>30</v>
       </c>
-      <c r="F26" t="s">
-        <v>47</v>
-      </c>
-      <c r="G26" t="s">
-        <v>51</v>
+      <c r="F26" s="16">
+        <v>0</v>
+      </c>
+      <c r="G26" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H26" t="s">
+        <v>51</v>
+      </c>
+      <c r="I26" t="s">
         <v>75</v>
       </c>
-      <c r="I26" t="s">
+      <c r="J26" t="s">
         <v>72</v>
       </c>
-      <c r="J26" s="13">
+      <c r="K26" s="13">
         <v>40</v>
       </c>
-      <c r="K26" t="s">
+      <c r="L26" t="s">
         <v>73</v>
       </c>
-      <c r="L26" t="s">
+      <c r="M26" t="s">
         <v>77</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2</v>
       </c>
@@ -1855,29 +1943,32 @@
       <c r="E27" t="s">
         <v>31</v>
       </c>
-      <c r="F27" t="s">
-        <v>47</v>
-      </c>
-      <c r="G27" t="s">
+      <c r="F27" s="16">
+        <v>0</v>
+      </c>
+      <c r="G27" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H27" t="s">
         <v>52</v>
       </c>
-      <c r="H27" t="s">
+      <c r="I27" t="s">
         <v>92</v>
       </c>
-      <c r="I27" t="s">
+      <c r="J27" t="s">
         <v>55</v>
       </c>
-      <c r="J27" s="13">
+      <c r="K27" s="13">
         <v>40</v>
       </c>
-      <c r="K27" t="s">
+      <c r="L27" t="s">
         <v>56</v>
       </c>
-      <c r="L27" t="s">
+      <c r="M27" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>2</v>
       </c>
@@ -1893,29 +1984,32 @@
       <c r="E28" t="s">
         <v>30</v>
       </c>
-      <c r="F28" t="s">
-        <v>47</v>
-      </c>
-      <c r="G28" t="s">
-        <v>51</v>
+      <c r="F28" s="16">
+        <v>0</v>
+      </c>
+      <c r="G28" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H28" t="s">
+        <v>51</v>
+      </c>
+      <c r="I28" t="s">
         <v>92</v>
       </c>
-      <c r="I28" t="s">
+      <c r="J28" t="s">
         <v>55</v>
       </c>
-      <c r="J28" s="13">
+      <c r="K28" s="13">
         <v>25</v>
       </c>
-      <c r="K28" t="s">
+      <c r="L28" t="s">
         <v>56</v>
       </c>
-      <c r="L28" t="s">
+      <c r="M28" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>2</v>
       </c>
@@ -1931,29 +2025,32 @@
       <c r="E29" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="F29" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G29" t="s">
-        <v>51</v>
+      <c r="F29" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G29" s="16">
+        <v>0.83333333333333337</v>
       </c>
       <c r="H29" t="s">
+        <v>51</v>
+      </c>
+      <c r="I29" t="s">
         <v>54</v>
       </c>
-      <c r="I29" t="s">
+      <c r="J29" t="s">
         <v>84</v>
       </c>
-      <c r="J29" s="13">
+      <c r="K29" s="13">
         <v>25</v>
       </c>
-      <c r="K29" t="s">
+      <c r="L29" t="s">
         <v>56</v>
       </c>
-      <c r="L29" t="s">
+      <c r="M29" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>2</v>
       </c>
@@ -1969,29 +2066,32 @@
       <c r="E30" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="F30" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="G30" t="s">
-        <v>51</v>
+      <c r="F30" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="G30" s="16">
+        <v>0.625</v>
       </c>
       <c r="H30" t="s">
+        <v>51</v>
+      </c>
+      <c r="I30" t="s">
         <v>54</v>
       </c>
-      <c r="I30" t="s">
+      <c r="J30" t="s">
         <v>84</v>
       </c>
-      <c r="J30" s="13">
+      <c r="K30" s="13">
         <v>30</v>
       </c>
-      <c r="K30" t="s">
+      <c r="L30" t="s">
         <v>56</v>
       </c>
-      <c r="L30" t="s">
+      <c r="M30" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>2</v>
       </c>
@@ -2007,29 +2107,32 @@
       <c r="E31" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F31" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="G31" t="s">
-        <v>51</v>
+      <c r="F31" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="G31" s="16">
+        <v>0.75</v>
       </c>
       <c r="H31" t="s">
+        <v>51</v>
+      </c>
+      <c r="I31" t="s">
         <v>54</v>
       </c>
-      <c r="I31" t="s">
+      <c r="J31" t="s">
         <v>84</v>
       </c>
-      <c r="J31" s="13">
+      <c r="K31" s="13">
         <v>20</v>
       </c>
-      <c r="K31" t="s">
+      <c r="L31" t="s">
         <v>56</v>
       </c>
-      <c r="L31" t="s">
+      <c r="M31" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>2</v>
       </c>
@@ -2045,29 +2148,32 @@
       <c r="E32" t="s">
         <v>32</v>
       </c>
-      <c r="F32" t="s">
-        <v>47</v>
-      </c>
-      <c r="G32" t="s">
-        <v>51</v>
+      <c r="F32" s="16">
+        <v>0</v>
+      </c>
+      <c r="G32" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H32" t="s">
+        <v>51</v>
+      </c>
+      <c r="I32" t="s">
         <v>92</v>
       </c>
-      <c r="I32" t="s">
+      <c r="J32" t="s">
         <v>55</v>
       </c>
-      <c r="J32" s="13">
+      <c r="K32" s="13">
         <v>20</v>
       </c>
-      <c r="K32" t="s">
+      <c r="L32" t="s">
         <v>56</v>
       </c>
-      <c r="L32" t="s">
+      <c r="M32" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>2</v>
       </c>
@@ -2083,29 +2189,32 @@
       <c r="E33" t="s">
         <v>36</v>
       </c>
-      <c r="F33" t="s">
-        <v>47</v>
-      </c>
-      <c r="G33" t="s">
-        <v>51</v>
+      <c r="F33" s="16">
+        <v>0</v>
+      </c>
+      <c r="G33" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H33" t="s">
+        <v>51</v>
+      </c>
+      <c r="I33" t="s">
         <v>92</v>
       </c>
-      <c r="I33" t="s">
+      <c r="J33" t="s">
         <v>55</v>
       </c>
-      <c r="J33" s="13">
+      <c r="K33" s="13">
         <v>20</v>
       </c>
-      <c r="K33" t="s">
+      <c r="L33" t="s">
         <v>56</v>
       </c>
-      <c r="L33" t="s">
+      <c r="M33" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>2</v>
       </c>
@@ -2121,29 +2230,32 @@
       <c r="E34" t="s">
         <v>42</v>
       </c>
-      <c r="F34" t="s">
-        <v>47</v>
-      </c>
-      <c r="G34" t="s">
+      <c r="F34" s="16">
+        <v>0</v>
+      </c>
+      <c r="G34" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H34" t="s">
         <v>53</v>
       </c>
-      <c r="H34" t="s">
+      <c r="I34" t="s">
         <v>92</v>
       </c>
-      <c r="I34" t="s">
+      <c r="J34" t="s">
         <v>55</v>
       </c>
-      <c r="J34" s="13">
+      <c r="K34" s="13">
         <v>30</v>
       </c>
-      <c r="K34" t="s">
+      <c r="L34" t="s">
         <v>56</v>
       </c>
-      <c r="L34" t="s">
+      <c r="M34" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>2</v>
       </c>
@@ -2159,29 +2271,32 @@
       <c r="E35" t="s">
         <v>31</v>
       </c>
-      <c r="F35" t="s">
-        <v>47</v>
-      </c>
-      <c r="G35" t="s">
+      <c r="F35" s="16">
+        <v>0</v>
+      </c>
+      <c r="G35" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H35" t="s">
         <v>52</v>
       </c>
-      <c r="H35" t="s">
+      <c r="I35" t="s">
         <v>92</v>
       </c>
-      <c r="I35" t="s">
+      <c r="J35" t="s">
         <v>55</v>
       </c>
-      <c r="J35" s="13">
+      <c r="K35" s="13">
         <v>70</v>
       </c>
-      <c r="K35" t="s">
+      <c r="L35" t="s">
         <v>56</v>
       </c>
-      <c r="L35" t="s">
+      <c r="M35" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>2</v>
       </c>
@@ -2197,29 +2312,32 @@
       <c r="E36" t="s">
         <v>45</v>
       </c>
-      <c r="F36" t="s">
-        <v>50</v>
-      </c>
-      <c r="G36" t="s">
-        <v>51</v>
+      <c r="F36" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G36" s="16">
+        <v>0.75</v>
       </c>
       <c r="H36" t="s">
+        <v>51</v>
+      </c>
+      <c r="I36" t="s">
         <v>93</v>
       </c>
-      <c r="I36" t="s">
+      <c r="J36" t="s">
         <v>56</v>
       </c>
-      <c r="J36" s="13">
-        <v>0</v>
-      </c>
-      <c r="K36" t="s">
+      <c r="K36" s="13">
+        <v>0</v>
+      </c>
+      <c r="L36" t="s">
         <v>56</v>
       </c>
-      <c r="L36" t="s">
+      <c r="M36" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>2</v>
       </c>
@@ -2235,29 +2353,32 @@
       <c r="E37" t="s">
         <v>45</v>
       </c>
-      <c r="F37" t="s">
-        <v>50</v>
-      </c>
-      <c r="G37" t="s">
-        <v>51</v>
+      <c r="F37" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G37" s="16">
+        <v>0.75</v>
       </c>
       <c r="H37" t="s">
+        <v>51</v>
+      </c>
+      <c r="I37" t="s">
         <v>93</v>
       </c>
-      <c r="I37" t="s">
+      <c r="J37" t="s">
         <v>56</v>
       </c>
-      <c r="J37" s="13">
+      <c r="K37" s="13">
         <v>20</v>
       </c>
-      <c r="K37" t="s">
+      <c r="L37" t="s">
         <v>56</v>
       </c>
-      <c r="L37" t="s">
+      <c r="M37" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>2</v>
       </c>
@@ -2273,29 +2394,32 @@
       <c r="E38" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="F38" s="12" t="s">
-        <v>85</v>
-      </c>
-      <c r="G38" t="s">
-        <v>51</v>
+      <c r="F38" s="17">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G38" s="16">
+        <v>0.83333333333333337</v>
       </c>
       <c r="H38" t="s">
+        <v>51</v>
+      </c>
+      <c r="I38" t="s">
         <v>54</v>
       </c>
-      <c r="I38" t="s">
+      <c r="J38" t="s">
         <v>84</v>
       </c>
-      <c r="J38" s="13">
+      <c r="K38" s="13">
         <v>30</v>
       </c>
-      <c r="K38" t="s">
+      <c r="L38" t="s">
         <v>56</v>
       </c>
-      <c r="L38" t="s">
+      <c r="M38" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>2</v>
       </c>
@@ -2311,29 +2435,32 @@
       <c r="E39" s="12" t="s">
         <v>82</v>
       </c>
-      <c r="F39" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="G39" t="s">
-        <v>51</v>
+      <c r="F39" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="G39" s="16">
+        <v>0.625</v>
       </c>
       <c r="H39" t="s">
+        <v>51</v>
+      </c>
+      <c r="I39" t="s">
         <v>54</v>
       </c>
-      <c r="I39" t="s">
+      <c r="J39" t="s">
         <v>84</v>
       </c>
-      <c r="J39" s="13">
+      <c r="K39" s="13">
         <v>35</v>
       </c>
-      <c r="K39" t="s">
+      <c r="L39" t="s">
         <v>56</v>
       </c>
-      <c r="L39" t="s">
+      <c r="M39" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A40">
         <v>2</v>
       </c>
@@ -2349,29 +2476,32 @@
       <c r="E40" s="12" t="s">
         <v>90</v>
       </c>
-      <c r="F40" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="G40" t="s">
-        <v>51</v>
+      <c r="F40" s="17">
+        <v>0.375</v>
+      </c>
+      <c r="G40" s="16">
+        <v>0.75</v>
       </c>
       <c r="H40" t="s">
+        <v>51</v>
+      </c>
+      <c r="I40" t="s">
         <v>54</v>
       </c>
-      <c r="I40" t="s">
+      <c r="J40" t="s">
         <v>84</v>
       </c>
-      <c r="J40" s="13">
+      <c r="K40" s="13">
         <v>35</v>
       </c>
-      <c r="K40" t="s">
+      <c r="L40" t="s">
         <v>56</v>
       </c>
-      <c r="L40" t="s">
+      <c r="M40" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>2</v>
       </c>
@@ -2387,29 +2517,32 @@
       <c r="E41" t="s">
         <v>43</v>
       </c>
-      <c r="F41" t="s">
-        <v>47</v>
-      </c>
-      <c r="G41" t="s">
-        <v>51</v>
+      <c r="F41" s="16">
+        <v>0</v>
+      </c>
+      <c r="G41" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H41" t="s">
+        <v>51</v>
+      </c>
+      <c r="I41" t="s">
         <v>92</v>
       </c>
-      <c r="I41" t="s">
+      <c r="J41" t="s">
         <v>55</v>
       </c>
-      <c r="J41" s="13">
+      <c r="K41" s="13">
         <v>35</v>
       </c>
-      <c r="K41" t="s">
+      <c r="L41" t="s">
         <v>56</v>
       </c>
-      <c r="L41" t="s">
+      <c r="M41" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>2</v>
       </c>
@@ -2425,29 +2558,32 @@
       <c r="E42" t="s">
         <v>32</v>
       </c>
-      <c r="F42" t="s">
-        <v>47</v>
-      </c>
-      <c r="G42" t="s">
-        <v>51</v>
+      <c r="F42" s="16">
+        <v>0</v>
+      </c>
+      <c r="G42" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H42" t="s">
+        <v>51</v>
+      </c>
+      <c r="I42" t="s">
         <v>92</v>
       </c>
-      <c r="I42" t="s">
+      <c r="J42" t="s">
         <v>55</v>
       </c>
-      <c r="J42" s="13">
+      <c r="K42" s="13">
         <v>60</v>
       </c>
-      <c r="K42" t="s">
+      <c r="L42" t="s">
         <v>55</v>
       </c>
-      <c r="L42" t="s">
+      <c r="M42" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>2</v>
       </c>
@@ -2463,29 +2599,32 @@
       <c r="E43" t="s">
         <v>29</v>
       </c>
-      <c r="F43" t="s">
-        <v>47</v>
-      </c>
-      <c r="G43" t="s">
-        <v>51</v>
+      <c r="F43" s="16">
+        <v>0</v>
+      </c>
+      <c r="G43" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H43" t="s">
+        <v>51</v>
+      </c>
+      <c r="I43" t="s">
         <v>92</v>
       </c>
-      <c r="I43" t="s">
+      <c r="J43" t="s">
         <v>55</v>
       </c>
-      <c r="J43" s="13">
+      <c r="K43" s="13">
         <v>70</v>
       </c>
-      <c r="K43" t="s">
+      <c r="L43" t="s">
         <v>55</v>
       </c>
-      <c r="L43" t="s">
+      <c r="M43" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>2</v>
       </c>
@@ -2501,29 +2640,32 @@
       <c r="E44" t="s">
         <v>29</v>
       </c>
-      <c r="F44" t="s">
-        <v>47</v>
-      </c>
-      <c r="G44" t="s">
-        <v>51</v>
+      <c r="F44" s="16">
+        <v>0</v>
+      </c>
+      <c r="G44" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H44" t="s">
+        <v>51</v>
+      </c>
+      <c r="I44" t="s">
         <v>92</v>
       </c>
-      <c r="I44" t="s">
+      <c r="J44" t="s">
         <v>55</v>
       </c>
-      <c r="J44" s="13">
-        <v>0</v>
-      </c>
-      <c r="K44" t="s">
+      <c r="K44" s="13">
+        <v>0</v>
+      </c>
+      <c r="L44" t="s">
         <v>55</v>
       </c>
-      <c r="L44" t="s">
+      <c r="M44" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>2</v>
       </c>
@@ -2539,29 +2681,32 @@
       <c r="E45" t="s">
         <v>31</v>
       </c>
-      <c r="F45" t="s">
-        <v>47</v>
-      </c>
-      <c r="G45" t="s">
+      <c r="F45" s="16">
+        <v>0</v>
+      </c>
+      <c r="G45" s="16">
+        <v>0.99930555555555556</v>
+      </c>
+      <c r="H45" t="s">
         <v>52</v>
       </c>
-      <c r="H45" t="s">
+      <c r="I45" t="s">
         <v>92</v>
       </c>
-      <c r="I45" t="s">
+      <c r="J45" t="s">
         <v>55</v>
       </c>
-      <c r="J45" s="13">
+      <c r="K45" s="13">
         <v>40</v>
       </c>
-      <c r="K45" t="s">
+      <c r="L45" t="s">
         <v>55</v>
       </c>
-      <c r="L45" t="s">
+      <c r="M45" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>2</v>
       </c>
@@ -2577,29 +2722,32 @@
       <c r="E46" t="s">
         <v>45</v>
       </c>
-      <c r="F46" t="s">
-        <v>50</v>
-      </c>
-      <c r="G46" t="s">
-        <v>51</v>
+      <c r="F46" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G46" s="16">
+        <v>0.75</v>
       </c>
       <c r="H46" t="s">
+        <v>51</v>
+      </c>
+      <c r="I46" t="s">
         <v>93</v>
       </c>
-      <c r="I46" t="s">
+      <c r="J46" t="s">
         <v>56</v>
       </c>
-      <c r="J46" s="13">
+      <c r="K46" s="13">
         <v>45</v>
       </c>
-      <c r="K46" t="s">
+      <c r="L46" t="s">
         <v>55</v>
       </c>
-      <c r="L46" t="s">
+      <c r="M46" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>2</v>
       </c>
@@ -2615,29 +2763,32 @@
       <c r="E47" t="s">
         <v>43</v>
       </c>
-      <c r="F47" t="s">
-        <v>47</v>
-      </c>
-      <c r="G47" t="s">
-        <v>51</v>
+      <c r="F47" s="16">
+        <v>0</v>
+      </c>
+      <c r="G47" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H47" t="s">
+        <v>51</v>
+      </c>
+      <c r="I47" t="s">
         <v>92</v>
       </c>
-      <c r="I47" t="s">
+      <c r="J47" t="s">
         <v>55</v>
       </c>
-      <c r="J47" s="13">
+      <c r="K47" s="13">
         <v>20</v>
       </c>
-      <c r="K47" t="s">
+      <c r="L47" t="s">
         <v>55</v>
       </c>
-      <c r="L47" t="s">
+      <c r="M47" t="s">
         <v>88</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>2</v>
       </c>
@@ -2653,29 +2804,32 @@
       <c r="E48" t="s">
         <v>45</v>
       </c>
-      <c r="F48" t="s">
-        <v>50</v>
-      </c>
-      <c r="G48" t="s">
-        <v>51</v>
+      <c r="F48" s="16">
+        <v>0.33333333333333331</v>
+      </c>
+      <c r="G48" s="16">
+        <v>0.75</v>
       </c>
       <c r="H48" t="s">
+        <v>51</v>
+      </c>
+      <c r="I48" t="s">
         <v>93</v>
       </c>
-      <c r="I48" t="s">
+      <c r="J48" t="s">
         <v>56</v>
       </c>
-      <c r="J48" s="13">
+      <c r="K48" s="13">
         <v>25</v>
       </c>
-      <c r="K48" t="s">
+      <c r="L48" t="s">
         <v>55</v>
       </c>
-      <c r="L48" t="s">
+      <c r="M48" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>2</v>
       </c>
@@ -2691,29 +2845,32 @@
       <c r="E49" t="s">
         <v>46</v>
       </c>
-      <c r="F49" t="s">
-        <v>47</v>
-      </c>
-      <c r="G49" t="s">
-        <v>51</v>
+      <c r="F49" s="16">
+        <v>0</v>
+      </c>
+      <c r="G49" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H49" t="s">
+        <v>51</v>
+      </c>
+      <c r="I49" t="s">
         <v>92</v>
       </c>
-      <c r="I49" t="s">
+      <c r="J49" t="s">
         <v>55</v>
       </c>
-      <c r="J49" s="13">
+      <c r="K49" s="13">
         <v>25</v>
       </c>
-      <c r="K49" t="s">
+      <c r="L49" t="s">
         <v>55</v>
       </c>
-      <c r="L49" t="s">
+      <c r="M49" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>2</v>
       </c>
@@ -2729,29 +2886,32 @@
       <c r="E50" t="s">
         <v>33</v>
       </c>
-      <c r="F50" t="s">
-        <v>48</v>
-      </c>
-      <c r="G50" t="s">
-        <v>51</v>
+      <c r="F50" s="16">
+        <v>0.375</v>
+      </c>
+      <c r="G50" s="16">
+        <v>0.70833333333333337</v>
       </c>
       <c r="H50" t="s">
+        <v>51</v>
+      </c>
+      <c r="I50" t="s">
         <v>93</v>
       </c>
-      <c r="I50" t="s">
+      <c r="J50" t="s">
         <v>56</v>
       </c>
-      <c r="J50" s="13">
+      <c r="K50" s="13">
         <v>15</v>
       </c>
-      <c r="K50" t="s">
+      <c r="L50" t="s">
         <v>55</v>
       </c>
-      <c r="L50" t="s">
+      <c r="M50" t="s">
         <v>87</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>2</v>
       </c>
@@ -2767,35 +2927,38 @@
       <c r="E51" t="s">
         <v>44</v>
       </c>
-      <c r="F51" t="s">
-        <v>47</v>
-      </c>
-      <c r="G51" t="s">
-        <v>51</v>
+      <c r="F51" s="16">
+        <v>0</v>
+      </c>
+      <c r="G51" s="16">
+        <v>0.99930555555555556</v>
       </c>
       <c r="H51" t="s">
+        <v>51</v>
+      </c>
+      <c r="I51" t="s">
         <v>92</v>
       </c>
-      <c r="I51" t="s">
+      <c r="J51" t="s">
         <v>55</v>
       </c>
-      <c r="J51" s="13">
+      <c r="K51" s="13">
         <v>35</v>
       </c>
-      <c r="K51" t="s">
+      <c r="L51" t="s">
         <v>55</v>
       </c>
-      <c r="L51" t="s">
+      <c r="M51" t="s">
         <v>86</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:13" x14ac:dyDescent="0.35">
       <c r="B52" s="13"/>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:13" x14ac:dyDescent="0.35">
       <c r="H53" s="15"/>
     </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:13" x14ac:dyDescent="0.35">
       <c r="H58" s="15"/>
     </row>
     <row r="69" spans="9:11" x14ac:dyDescent="0.35">
@@ -3022,7 +3185,7 @@
     <row r="604" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K604">
         <f>COUNTIF(K2:K601, "Sí")</f>
-        <v>15</v>
+        <v>0</v>
       </c>
     </row>
     <row r="605" spans="11:11" x14ac:dyDescent="0.35">
@@ -3033,7 +3196,7 @@
     <row r="606" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K606">
         <f>COUNTIF(K2:K601, "No")</f>
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="608" spans="11:11" x14ac:dyDescent="0.35">
@@ -3042,9 +3205,9 @@
       </c>
     </row>
     <row r="609" spans="11:11" x14ac:dyDescent="0.35">
-      <c r="K609" s="4">
+      <c r="K609" s="4" t="e">
         <f>COUNTIF(K2:K601, "Sí") / (COUNTIF(K2:K601, "Sí") + COUNTIF(K2:K601, "No")) * 100</f>
-        <v>60</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="611" spans="11:11" x14ac:dyDescent="0.35">
@@ -3075,7 +3238,7 @@
     <row r="617" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K617">
         <f>COUNTIF(H2:H601, "Alta")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="618" spans="11:11" x14ac:dyDescent="0.35">
@@ -3086,7 +3249,7 @@
     <row r="619" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K619">
         <f>COUNTIFS(H2:H601, "Alta", K2:K601, "Sí")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="620" spans="11:11" x14ac:dyDescent="0.35">
@@ -3095,9 +3258,9 @@
       </c>
     </row>
     <row r="621" spans="11:11" x14ac:dyDescent="0.35">
-      <c r="K621">
+      <c r="K621" t="e">
         <f>COUNTIFS(H2:H601, "Alta", K2:K601, "Sí") / COUNTIF(H2:H601, "Alta") * 100</f>
-        <v>100</v>
+        <v>#DIV/0!</v>
       </c>
     </row>
     <row r="623" spans="11:11" x14ac:dyDescent="0.35">
@@ -3119,7 +3282,7 @@
     <row r="627" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K627" s="9">
         <f>COUNTIF(G2:G601, "Centro")</f>
-        <v>37</v>
+        <v>0</v>
       </c>
     </row>
     <row r="628" spans="11:11" x14ac:dyDescent="0.35">
@@ -3130,7 +3293,7 @@
     <row r="629" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K629" s="9">
         <f>COUNTIF(G2:G601, "Norte")</f>
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="630" spans="11:11" x14ac:dyDescent="0.35">
@@ -3141,7 +3304,7 @@
     <row r="631" spans="11:11" x14ac:dyDescent="0.35">
       <c r="K631" s="9">
         <f>COUNTIF(G2:G601, "Poniente")</f>
-        <v>7</v>
+        <v>0</v>
       </c>
     </row>
     <row r="632" spans="11:11" x14ac:dyDescent="0.35">

</xml_diff>